<commit_message>
260724 update on LR draft
</commit_message>
<xml_diff>
--- a/Projects/MISQ/MISQ round 2/afterSEmeeting260719.xlsx
+++ b/Projects/MISQ/MISQ round 2/afterSEmeeting260719.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanchen/Desktop/geek-community/Projects/MISQ/MISQ round 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54313D65-FEB8-B441-8ECD-A6E7EBC7CAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319CF024-094B-4344-A521-29941CA66979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="38240" windowHeight="19320" activeTab="4" xr2:uid="{30F402B7-E6D8-E34B-8063-713AC97DE139}"/>
+    <workbookView xWindow="80" yWindow="660" windowWidth="38160" windowHeight="19420" activeTab="4" xr2:uid="{30F402B7-E6D8-E34B-8063-713AC97DE139}"/>
   </bookViews>
   <sheets>
     <sheet name="main results" sheetId="19" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="403">
   <si>
     <t>-0.046 ***</t>
   </si>
@@ -1367,9 +1367,6 @@
     <t>GenAI Effect</t>
   </si>
   <si>
-    <t>Borwankar et al., 2023</t>
-  </si>
-  <si>
     <t>Stack Overflow</t>
   </si>
   <si>
@@ -1388,15 +1385,9 @@
     <t>answer-user-day</t>
   </si>
   <si>
-    <t>Make answers shorter, more negative and harder to read</t>
-  </si>
-  <si>
     <t>Decrease # of likes</t>
   </si>
   <si>
-    <t>Burtch et al., 2023</t>
-  </si>
-  <si>
     <t>GenAI introduction</t>
   </si>
   <si>
@@ -1409,36 +1400,21 @@
     <t>Reduce # of questions</t>
   </si>
   <si>
-    <t>del Rio-Chanona et al., 2023</t>
-  </si>
-  <si>
-    <t>Quinn &amp; Gutt, 2023</t>
-  </si>
-  <si>
     <t>Stack Exchange</t>
   </si>
   <si>
-    <t>Sanatizadeh et al., 2023</t>
-  </si>
-  <si>
     <t>Questioner, Answerer, Viewer</t>
   </si>
   <si>
     <t>post-day</t>
   </si>
   <si>
-    <t>Reduce # of questions; make questions more difficult to read</t>
-  </si>
-  <si>
     <t>Reduce # of answers; make answers longer, more difficult to read</t>
   </si>
   <si>
     <t>Reduce # of views; increase # of likes</t>
   </si>
   <si>
-    <t>Shan &amp; Qiu, 2023</t>
-  </si>
-  <si>
     <t>Answerer</t>
   </si>
   <si>
@@ -1448,9 +1424,6 @@
     <t>Increase # of answers; make answers shorter and easier to read</t>
   </si>
   <si>
-    <t>Su et al., 2023</t>
-  </si>
-  <si>
     <t>Quora</t>
   </si>
   <si>
@@ -1460,30 +1433,15 @@
     <t>question-week</t>
   </si>
   <si>
-    <t>Increase # of answers; make answers longer and similar to AI answers</t>
-  </si>
-  <si>
-    <t>Xue et al., 2023</t>
-  </si>
-  <si>
     <t>topic-day</t>
   </si>
   <si>
-    <t>Reduce # of questions; make questions longer, more difficult to read</t>
-  </si>
-  <si>
-    <t>Li &amp; Kim, 2024</t>
-  </si>
-  <si>
     <t>Reduce # of answers</t>
   </si>
   <si>
     <t>Reduce # of likes</t>
   </si>
   <si>
-    <t>Wang &amp; Zheng, 2024</t>
-  </si>
-  <si>
     <t>Increase # of questions</t>
   </si>
   <si>
@@ -1494,12 +1452,6 @@
   </si>
   <si>
     <t>Reduce # of questions; make questions higher quality (simpler questions disappear)</t>
-  </si>
-  <si>
-    <t>Increase question quality</t>
-  </si>
-  <si>
-    <t>AI label versus. AI content?</t>
   </si>
   <si>
     <t>Difference from external GenAI research</t>
@@ -1715,12 +1667,268 @@
   <si>
     <t>outline (wondering) -&gt; AI</t>
   </si>
+  <si>
+    <t>Borwankar et al. (2026)</t>
+  </si>
+  <si>
+    <t>del Rio-Chanona et al. (2024)</t>
+  </si>
+  <si>
+    <t>Quinn &amp; Gutt (2025)</t>
+  </si>
+  <si>
+    <t>Xue et al. (2026)</t>
+  </si>
+  <si>
+    <t>Shan &amp; Qiu  (2026)</t>
+  </si>
+  <si>
+    <t>Fang &amp; Zhou (2026)</t>
+  </si>
+  <si>
+    <t>Zhihu</t>
+  </si>
+  <si>
+    <t>user-month</t>
+  </si>
+  <si>
+    <t>Increase # answers; make answer shorter</t>
+  </si>
+  <si>
+    <t>Increase # views</t>
+  </si>
+  <si>
+    <t>Rao et al, (2026)</t>
+  </si>
+  <si>
+    <t>Questioner, Viewer</t>
+  </si>
+  <si>
+    <t>user-week</t>
+  </si>
+  <si>
+    <t>Increase # of questions; make questions longer, more novel; Increase # of upvotes of questions</t>
+  </si>
+  <si>
+    <t>Su et al. (2025)</t>
+  </si>
+  <si>
+    <t>Increase # of answers; make answers</t>
+  </si>
+  <si>
+    <t>longer and similar to AI answers</t>
+  </si>
+  <si>
+    <t>Make answers shorter, more negative and easier to read</t>
+  </si>
+  <si>
+    <t>Reduce # of questions; make questions more complex and higher-quality</t>
+  </si>
+  <si>
+    <t>Burtch et al. (2024)</t>
+  </si>
+  <si>
+    <t>Sanatizadeh et al. (2025)</t>
+  </si>
+  <si>
+    <t>Li &amp; Kim (2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wang &amp; Zheng (2024) </t>
+  </si>
+  <si>
+    <t>Key Findings</t>
+  </si>
+  <si>
+    <t>Technical</t>
+  </si>
+  <si>
+    <t>Natural Exp.</t>
+  </si>
+  <si>
+    <t>↓ answers; ↓ likes</t>
+  </si>
+  <si>
+    <t>↓ questions; remaining questions ↑ quality</t>
+  </si>
+  <si>
+    <t>↑ answers; answers shorter &amp; easier to read</t>
+  </si>
+  <si>
+    <t>Rao et al. (2026)</t>
+  </si>
+  <si>
+    <t>↑ questions; questions longer, more novel; ↑ upvotes</t>
+  </si>
+  <si>
+    <t>Wang &amp; Zheng (2024)</t>
+  </si>
+  <si>
+    <t>↑ questions; ↑ answers &amp; acceptance; ↑ views</t>
+  </si>
+  <si>
+    <t>Answers shorter, more negative; ↓ likes</t>
+  </si>
+  <si>
+    <t>External GenAI · General Community</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>↑ answers; answers shorter; ↑ views</t>
+  </si>
+  <si>
+    <t>NE + Experiment</t>
+  </si>
+  <si>
+    <t>Community Domain</t>
+  </si>
+  <si>
+    <t>SegmentFault</t>
+  </si>
+  <si>
+    <t>External GenAI · Technical Community · Introduction of ChatGPT</t>
+  </si>
+  <si>
+    <t>External GenAI · Technical Community · Ban ChatGPT</t>
+  </si>
+  <si>
+    <t>question</t>
+  </si>
+  <si>
+    <t>Our Study (2026)</t>
+  </si>
+  <si>
+    <t>Mechanism Identified</t>
+  </si>
+  <si>
+    <t>Shan &amp; Qiu (2026, ISR)</t>
+  </si>
+  <si>
+    <t>Xue et al. (2026, ISR)</t>
+  </si>
+  <si>
+    <t>Quinn &amp; Gutt (2025, JMIS)</t>
+  </si>
+  <si>
+    <t>Sanatizadeh et al. (2025, I&amp;M)</t>
+  </si>
+  <si>
+    <t>Fang &amp; Zhou (2026, I&amp;M)</t>
+  </si>
+  <si>
+    <t>AI label → weak competitor perception
+AI length/quality → signal comprehensiveness → deter contribution 
+AI quality → make human differentiate → boost quality</t>
+  </si>
+  <si>
+    <t>AI label effect → boost contribution willing
+AI Conformity → increased human-AI similarity → increased length</t>
+  </si>
+  <si>
+    <t>↑ answers; ↑ answer length</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>How AI answers provided</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Panel A: Research on The Impact of External GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Panel B: Research on The Impact of External GenAI</t>
+  </si>
+  <si>
+    <t>AI label v.s. 
+AI content?</t>
+  </si>
+  <si>
+    <t>↓ answers; ↑ answers quality</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">provided to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>existing questions</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> through batch processing</t>
+    </r>
+  </si>
+  <si>
+    <t>Randomized Exp.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">randomly provided to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>new questions</t>
+    </r>
+  </si>
+  <si>
+    <t>Natural Exp. + Experiment</t>
+  </si>
+  <si>
+    <t>Topic-Week</t>
+  </si>
+  <si>
+    <t>Post-Day</t>
+  </si>
+  <si>
+    <t>User-Day</t>
+  </si>
+  <si>
+    <t>User-Week</t>
+  </si>
+  <si>
+    <t>Topic-Day</t>
+  </si>
+  <si>
+    <t>Answer-User-Day</t>
+  </si>
+  <si>
+    <t>User-Month</t>
+  </si>
+  <si>
+    <t>Question-Week</t>
+  </si>
+  <si>
+    <t>↓ Questions</t>
+  </si>
+  <si>
+    <t>↓ Questions; remaining questions more complex &amp; higher quality; ↓ answers; answers longer &amp; harder to read; ↓ views; ↑ likes</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1878,12 +2086,6 @@
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -1901,6 +2103,38 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFB45309"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1910,7 +2144,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1988,11 +2222,77 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -2229,43 +2529,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2282,14 +2546,121 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3317,11 +3688,11 @@
         <v>54</v>
       </c>
       <c r="I2" s="9"/>
-      <c r="J2" s="97"/>
-      <c r="K2" s="98" t="s">
-        <v>318</v>
-      </c>
-      <c r="L2" s="98"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="86" t="s">
+        <v>302</v>
+      </c>
+      <c r="L2" s="86"/>
       <c r="N2" s="5" t="s">
         <v>202</v>
       </c>
@@ -3338,14 +3709,14 @@
         <v>126</v>
       </c>
       <c r="I3" s="9"/>
-      <c r="J3" s="99" t="s">
-        <v>319</v>
-      </c>
-      <c r="K3" s="100" t="s">
-        <v>320</v>
-      </c>
-      <c r="L3" s="101" t="s">
-        <v>321</v>
+      <c r="J3" s="87" t="s">
+        <v>303</v>
+      </c>
+      <c r="K3" s="88" t="s">
+        <v>304</v>
+      </c>
+      <c r="L3" s="89" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.2">
@@ -3359,12 +3730,12 @@
         <v>67</v>
       </c>
       <c r="H4" s="63"/>
-      <c r="J4" s="102"/>
-      <c r="K4" s="101" t="s">
+      <c r="J4" s="90"/>
+      <c r="K4" s="89" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="101" t="s">
-        <v>322</v>
+      <c r="L4" s="89" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.2">
@@ -3383,12 +3754,12 @@
       <c r="I5" t="s">
         <v>129</v>
       </c>
-      <c r="J5" s="99" t="s">
-        <v>323</v>
-      </c>
-      <c r="K5" s="101"/>
-      <c r="L5" s="101" t="s">
-        <v>324</v>
+      <c r="J5" s="87" t="s">
+        <v>307</v>
+      </c>
+      <c r="K5" s="89"/>
+      <c r="L5" s="89" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.2">
@@ -3405,9 +3776,9 @@
       <c r="I6" t="s">
         <v>130</v>
       </c>
-      <c r="J6" s="102"/>
-      <c r="K6" s="101"/>
-      <c r="L6" s="101" t="s">
+      <c r="J6" s="90"/>
+      <c r="K6" s="89"/>
+      <c r="L6" s="89" t="s">
         <v>35</v>
       </c>
     </row>
@@ -3427,12 +3798,12 @@
       <c r="I7" t="s">
         <v>131</v>
       </c>
-      <c r="J7" s="99" t="s">
-        <v>325</v>
-      </c>
-      <c r="K7" s="101"/>
-      <c r="L7" s="101" t="s">
-        <v>326</v>
+      <c r="J7" s="87" t="s">
+        <v>309</v>
+      </c>
+      <c r="K7" s="89"/>
+      <c r="L7" s="89" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
@@ -3449,9 +3820,9 @@
       <c r="I8" t="s">
         <v>132</v>
       </c>
-      <c r="J8" s="102"/>
-      <c r="K8" s="101"/>
-      <c r="L8" s="101" t="s">
+      <c r="J8" s="90"/>
+      <c r="K8" s="89"/>
+      <c r="L8" s="89" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3468,12 +3839,12 @@
       <c r="H9" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="J9" s="99" t="s">
-        <v>327</v>
-      </c>
-      <c r="K9" s="101"/>
-      <c r="L9" s="101" t="s">
-        <v>328</v>
+      <c r="J9" s="87" t="s">
+        <v>311</v>
+      </c>
+      <c r="K9" s="89"/>
+      <c r="L9" s="89" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.2">
@@ -3487,10 +3858,10 @@
       <c r="H10" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="J10" s="102"/>
-      <c r="K10" s="101"/>
-      <c r="L10" s="101" t="s">
-        <v>329</v>
+      <c r="J10" s="90"/>
+      <c r="K10" s="89"/>
+      <c r="L10" s="89" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.2">
@@ -3506,12 +3877,12 @@
       <c r="H11" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="J11" s="99" t="s">
-        <v>330</v>
-      </c>
-      <c r="K11" s="101"/>
-      <c r="L11" s="101" t="s">
-        <v>331</v>
+      <c r="J11" s="87" t="s">
+        <v>314</v>
+      </c>
+      <c r="K11" s="89"/>
+      <c r="L11" s="89" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.2">
@@ -3527,10 +3898,10 @@
       <c r="H12" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="J12" s="102"/>
-      <c r="K12" s="101"/>
-      <c r="L12" s="101" t="s">
-        <v>332</v>
+      <c r="J12" s="90"/>
+      <c r="K12" s="89"/>
+      <c r="L12" s="89" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.2">
@@ -3546,14 +3917,14 @@
       <c r="H13" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="J13" s="97" t="s">
-        <v>333</v>
-      </c>
-      <c r="K13" s="101" t="s">
-        <v>334</v>
-      </c>
-      <c r="L13" s="101" t="s">
-        <v>335</v>
+      <c r="J13" s="85" t="s">
+        <v>317</v>
+      </c>
+      <c r="K13" s="89" t="s">
+        <v>318</v>
+      </c>
+      <c r="L13" s="89" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.2">
@@ -5818,597 +6189,1106 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0063E07F-BB6D-304D-9967-A6255D4D21DE}">
-  <dimension ref="A2:J38"/>
+  <dimension ref="A1:P83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="48.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.1640625" customWidth="1"/>
-    <col min="4" max="4" width="22.1640625" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5" customWidth="1"/>
-    <col min="9" max="9" width="54.5" customWidth="1"/>
-    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" customWidth="1"/>
+    <col min="4" max="4" width="9.1640625" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="37.5" customWidth="1"/>
+    <col min="8" max="8" width="9.83203125" style="108" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="48.1640625" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="12" width="15.33203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="15" max="15" width="15.6640625" customWidth="1"/>
+    <col min="16" max="16" width="47.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B2" s="84" t="s">
+    <row r="1" spans="3:10" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="3:10" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="91" t="s">
         <v>261</v>
       </c>
-      <c r="C2" s="84" t="s">
+      <c r="D2" s="91" t="s">
         <v>262</v>
       </c>
-      <c r="D2" s="84" t="s">
+      <c r="E2" s="91" t="s">
         <v>263</v>
       </c>
-      <c r="E2" s="84" t="s">
+      <c r="F2" s="91" t="s">
         <v>264</v>
       </c>
-      <c r="F2" s="84" t="s">
+      <c r="G2" s="91" t="s">
         <v>265</v>
       </c>
-      <c r="G2" s="84" t="s">
+      <c r="H2" s="91" t="s">
         <v>266</v>
       </c>
-      <c r="H2" s="84" t="s">
+      <c r="I2" s="91" t="s">
         <v>267</v>
       </c>
-      <c r="I2" s="84" t="s">
+      <c r="J2" s="91" t="s">
         <v>268</v>
       </c>
-      <c r="J2" s="96" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B3" s="85" t="s">
+    </row>
+    <row r="3" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C3" s="100" t="s">
+        <v>330</v>
+      </c>
+      <c r="D3" s="102" t="s">
         <v>269</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="E3" s="102" t="s">
         <v>270</v>
       </c>
-      <c r="D3" s="86" t="s">
+      <c r="F3" s="102" t="s">
         <v>271</v>
       </c>
-      <c r="E3" s="86" t="s">
+      <c r="G3" s="102" t="s">
         <v>272</v>
       </c>
-      <c r="F3" s="86" t="s">
+      <c r="H3" s="102" t="s">
         <v>273</v>
       </c>
-      <c r="G3" s="86" t="s">
+      <c r="I3" s="102" t="s">
         <v>274</v>
       </c>
-      <c r="H3" s="86" t="s">
+      <c r="J3" s="94" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="4" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C4" s="99"/>
+      <c r="D4" s="101"/>
+      <c r="E4" s="101"/>
+      <c r="F4" s="101"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="101"/>
+      <c r="I4" s="101"/>
+      <c r="J4" s="94" t="s">
         <v>275</v>
       </c>
-      <c r="I3" s="87" t="s">
+    </row>
+    <row r="5" spans="3:10" ht="26" x14ac:dyDescent="0.2">
+      <c r="C5" s="92" t="s">
+        <v>349</v>
+      </c>
+      <c r="D5" s="93" t="s">
+        <v>269</v>
+      </c>
+      <c r="E5" s="93" t="s">
+        <v>270</v>
+      </c>
+      <c r="F5" s="93" t="s">
         <v>276</v>
       </c>
-      <c r="J3" s="89" t="s">
+      <c r="G5" s="93" t="s">
+        <v>272</v>
+      </c>
+      <c r="H5" s="93" t="s">
+        <v>277</v>
+      </c>
+      <c r="I5" s="93" t="s">
+        <v>278</v>
+      </c>
+      <c r="J5" s="94" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="6" spans="3:10" ht="26" x14ac:dyDescent="0.2">
+      <c r="C6" s="92" t="s">
+        <v>331</v>
+      </c>
+      <c r="D6" s="93" t="s">
+        <v>269</v>
+      </c>
+      <c r="E6" s="93" t="s">
+        <v>270</v>
+      </c>
+      <c r="F6" s="93" t="s">
+        <v>276</v>
+      </c>
+      <c r="G6" s="93" t="s">
+        <v>272</v>
+      </c>
+      <c r="H6" s="93" t="s">
+        <v>277</v>
+      </c>
+      <c r="I6" s="93" t="s">
+        <v>278</v>
+      </c>
+      <c r="J6" s="94" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="7" spans="3:10" ht="26" x14ac:dyDescent="0.2">
+      <c r="C7" s="92" t="s">
+        <v>332</v>
+      </c>
+      <c r="D7" s="93" t="s">
+        <v>280</v>
+      </c>
+      <c r="E7" s="93" t="s">
+        <v>270</v>
+      </c>
+      <c r="F7" s="93" t="s">
+        <v>276</v>
+      </c>
+      <c r="G7" s="93" t="s">
+        <v>272</v>
+      </c>
+      <c r="H7" s="93" t="s">
+        <v>277</v>
+      </c>
+      <c r="I7" s="93" t="s">
+        <v>278</v>
+      </c>
+      <c r="J7" s="94" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="8" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C8" s="99" t="s">
+        <v>350</v>
+      </c>
+      <c r="D8" s="101" t="s">
+        <v>280</v>
+      </c>
+      <c r="E8" s="101" t="s">
+        <v>270</v>
+      </c>
+      <c r="F8" s="101" t="s">
+        <v>276</v>
+      </c>
+      <c r="G8" s="101" t="s">
+        <v>272</v>
+      </c>
+      <c r="H8" s="101" t="s">
+        <v>281</v>
+      </c>
+      <c r="I8" s="101" t="s">
+        <v>282</v>
+      </c>
+      <c r="J8" s="94" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="9" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C9" s="99"/>
+      <c r="D9" s="101"/>
+      <c r="E9" s="101"/>
+      <c r="F9" s="101"/>
+      <c r="G9" s="101"/>
+      <c r="H9" s="101"/>
+      <c r="I9" s="101"/>
+      <c r="J9" s="94" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="10" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C10" s="99"/>
+      <c r="D10" s="101"/>
+      <c r="E10" s="101"/>
+      <c r="F10" s="101"/>
+      <c r="G10" s="101"/>
+      <c r="H10" s="101"/>
+      <c r="I10" s="101"/>
+      <c r="J10" s="94" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="11" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C11" s="99" t="s">
+        <v>351</v>
+      </c>
+      <c r="D11" s="101" t="s">
+        <v>269</v>
+      </c>
+      <c r="E11" s="101" t="s">
+        <v>270</v>
+      </c>
+      <c r="F11" s="101" t="s">
+        <v>276</v>
+      </c>
+      <c r="G11" s="101" t="s">
+        <v>272</v>
+      </c>
+      <c r="H11" s="101" t="s">
+        <v>273</v>
+      </c>
+      <c r="I11" s="101" t="s">
+        <v>286</v>
+      </c>
+      <c r="J11" s="94" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="12" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C12" s="99"/>
+      <c r="D12" s="101"/>
+      <c r="E12" s="101"/>
+      <c r="F12" s="101"/>
+      <c r="G12" s="101"/>
+      <c r="H12" s="101"/>
+      <c r="I12" s="101"/>
+      <c r="J12" s="94" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="13" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C13" s="99" t="s">
+        <v>352</v>
+      </c>
+      <c r="D13" s="101" t="s">
+        <v>280</v>
+      </c>
+      <c r="E13" s="101" t="s">
+        <v>270</v>
+      </c>
+      <c r="F13" s="101" t="s">
+        <v>271</v>
+      </c>
+      <c r="G13" s="101" t="s">
+        <v>272</v>
+      </c>
+      <c r="H13" s="101" t="s">
+        <v>281</v>
+      </c>
+      <c r="I13" s="101" t="s">
+        <v>278</v>
+      </c>
+      <c r="J13" s="94" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="14" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C14" s="99"/>
+      <c r="D14" s="101"/>
+      <c r="E14" s="101"/>
+      <c r="F14" s="101"/>
+      <c r="G14" s="101"/>
+      <c r="H14" s="101"/>
+      <c r="I14" s="101"/>
+      <c r="J14" s="94" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="15" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C15" s="99"/>
+      <c r="D15" s="101"/>
+      <c r="E15" s="101"/>
+      <c r="F15" s="101"/>
+      <c r="G15" s="101"/>
+      <c r="H15" s="101"/>
+      <c r="I15" s="101"/>
+      <c r="J15" s="94" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="16" spans="3:10" ht="26" x14ac:dyDescent="0.2">
+      <c r="C16" s="95" t="s">
+        <v>333</v>
+      </c>
+      <c r="D16" s="96" t="s">
+        <v>269</v>
+      </c>
+      <c r="E16" s="96" t="s">
+        <v>270</v>
+      </c>
+      <c r="F16" s="96" t="s">
+        <v>276</v>
+      </c>
+      <c r="G16" s="96" t="s">
+        <v>272</v>
+      </c>
+      <c r="H16" s="96" t="s">
+        <v>277</v>
+      </c>
+      <c r="I16" s="96" t="s">
+        <v>291</v>
+      </c>
+      <c r="J16" s="94" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="26" x14ac:dyDescent="0.2">
+      <c r="C17" s="92" t="s">
+        <v>334</v>
+      </c>
+      <c r="D17" s="96" t="s">
+        <v>269</v>
+      </c>
+      <c r="E17" s="96" t="s">
+        <v>270</v>
+      </c>
+      <c r="F17" s="96" t="s">
+        <v>276</v>
+      </c>
+      <c r="G17" s="96" t="s">
+        <v>272</v>
+      </c>
+      <c r="H17" s="96" t="s">
+        <v>285</v>
+      </c>
+      <c r="I17" s="96" t="s">
+        <v>286</v>
+      </c>
+      <c r="J17" s="94" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C18" s="99" t="s">
+        <v>335</v>
+      </c>
+      <c r="D18" s="103" t="s">
+        <v>336</v>
+      </c>
+      <c r="E18" s="103" t="s">
+        <v>270</v>
+      </c>
+      <c r="F18" s="103" t="s">
+        <v>271</v>
+      </c>
+      <c r="G18" s="104" t="s">
+        <v>272</v>
+      </c>
+      <c r="H18" s="103" t="s">
+        <v>273</v>
+      </c>
+      <c r="I18" s="103" t="s">
+        <v>337</v>
+      </c>
+      <c r="J18" s="94" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C19" s="99"/>
+      <c r="D19" s="103"/>
+      <c r="E19" s="103"/>
+      <c r="F19" s="103"/>
+      <c r="G19" s="104"/>
+      <c r="H19" s="103"/>
+      <c r="I19" s="103"/>
+      <c r="J19" s="94" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="26" x14ac:dyDescent="0.2">
+      <c r="C20" s="92" t="s">
+        <v>340</v>
+      </c>
+      <c r="D20" s="97" t="s">
+        <v>269</v>
+      </c>
+      <c r="E20" s="97" t="s">
+        <v>270</v>
+      </c>
+      <c r="F20" s="97" t="s">
+        <v>276</v>
+      </c>
+      <c r="G20" s="97" t="s">
+        <v>272</v>
+      </c>
+      <c r="H20" s="97" t="s">
+        <v>341</v>
+      </c>
+      <c r="I20" s="96" t="s">
+        <v>342</v>
+      </c>
+      <c r="J20" s="94" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C21" s="99" t="s">
+        <v>344</v>
+      </c>
+      <c r="D21" s="101" t="s">
+        <v>288</v>
+      </c>
+      <c r="E21" s="101" t="s">
+        <v>289</v>
+      </c>
+      <c r="F21" s="101" t="s">
+        <v>276</v>
+      </c>
+      <c r="G21" s="101" t="s">
+        <v>272</v>
+      </c>
+      <c r="H21" s="101" t="s">
+        <v>285</v>
+      </c>
+      <c r="I21" s="101" t="s">
+        <v>290</v>
+      </c>
+      <c r="J21" s="94" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="105"/>
+      <c r="D22" s="106"/>
+      <c r="E22" s="106"/>
+      <c r="F22" s="106"/>
+      <c r="G22" s="106"/>
+      <c r="H22" s="106"/>
+      <c r="I22" s="106"/>
+      <c r="J22" s="98" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>298</v>
+      </c>
+      <c r="B29" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B30" s="84" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>299</v>
+      </c>
+      <c r="B31" s="84" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B32" s="84" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B33" s="84" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>323</v>
+      </c>
+      <c r="C39" t="s">
+        <v>324</v>
+      </c>
+      <c r="D39" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="D40" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C41" t="s">
+        <v>327</v>
+      </c>
+      <c r="D41" t="s">
+        <v>329</v>
+      </c>
+      <c r="E41" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C42" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B45" s="109" t="s">
+        <v>385</v>
+      </c>
+      <c r="C45" s="109"/>
+      <c r="D45" s="109"/>
+      <c r="E45" s="109"/>
+      <c r="F45" s="109"/>
+      <c r="G45" s="109"/>
+      <c r="H45" s="109"/>
+    </row>
+    <row r="46" spans="2:8" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B46" s="110" t="s">
+        <v>261</v>
+      </c>
+      <c r="C46" s="110" t="s">
+        <v>262</v>
+      </c>
+      <c r="D46" s="111" t="s">
+        <v>368</v>
+      </c>
+      <c r="E46" s="111" t="s">
+        <v>265</v>
+      </c>
+      <c r="F46" s="110" t="s">
+        <v>267</v>
+      </c>
+      <c r="G46" s="110" t="s">
+        <v>353</v>
+      </c>
+      <c r="H46" s="112" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="47" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B47" s="113" t="s">
+        <v>370</v>
+      </c>
+      <c r="C47" s="113"/>
+      <c r="D47" s="113"/>
+      <c r="E47" s="113"/>
+      <c r="F47" s="113"/>
+      <c r="G47" s="113"/>
+      <c r="H47" s="113"/>
+    </row>
+    <row r="48" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B48" s="114" t="s">
+        <v>349</v>
+      </c>
+      <c r="C48" s="114" t="s">
+        <v>269</v>
+      </c>
+      <c r="D48" s="114" t="s">
+        <v>354</v>
+      </c>
+      <c r="E48" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F48" s="114" t="s">
+        <v>393</v>
+      </c>
+      <c r="G48" s="114" t="s">
+        <v>401</v>
+      </c>
+      <c r="H48" s="115" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B4" s="85"/>
-      <c r="C4" s="86"/>
-      <c r="D4" s="86"/>
-      <c r="E4" s="86"/>
-      <c r="F4" s="86"/>
-      <c r="G4" s="86"/>
-      <c r="H4" s="86"/>
-      <c r="I4" s="87" t="s">
-        <v>277</v>
-      </c>
-      <c r="J4" s="89" t="s">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B49" s="114" t="s">
+        <v>331</v>
+      </c>
+      <c r="C49" s="114" t="s">
+        <v>269</v>
+      </c>
+      <c r="D49" s="114" t="s">
+        <v>354</v>
+      </c>
+      <c r="E49" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F49" s="114" t="s">
+        <v>393</v>
+      </c>
+      <c r="G49" s="114" t="s">
+        <v>401</v>
+      </c>
+      <c r="H49" s="115" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B5" s="88" t="s">
-        <v>278</v>
-      </c>
-      <c r="C5" s="89" t="s">
-        <v>270</v>
-      </c>
-      <c r="D5" s="89" t="s">
-        <v>271</v>
-      </c>
-      <c r="E5" s="89" t="s">
-        <v>279</v>
-      </c>
-      <c r="F5" s="89" t="s">
-        <v>273</v>
-      </c>
-      <c r="G5" s="89" t="s">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B50" s="114" t="s">
+        <v>377</v>
+      </c>
+      <c r="C50" s="114" t="s">
         <v>280</v>
       </c>
-      <c r="H5" s="89" t="s">
-        <v>281</v>
-      </c>
-      <c r="I5" s="87" t="s">
-        <v>282</v>
-      </c>
-      <c r="J5" s="89" t="s">
+      <c r="D50" s="114" t="s">
+        <v>354</v>
+      </c>
+      <c r="E50" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F50" s="114" t="s">
+        <v>393</v>
+      </c>
+      <c r="G50" s="114" t="s">
+        <v>401</v>
+      </c>
+      <c r="H50" s="115" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B6" s="88" t="s">
-        <v>283</v>
-      </c>
-      <c r="C6" s="89" t="s">
-        <v>270</v>
-      </c>
-      <c r="D6" s="89" t="s">
-        <v>271</v>
-      </c>
-      <c r="E6" s="89" t="s">
-        <v>279</v>
-      </c>
-      <c r="F6" s="89" t="s">
-        <v>273</v>
-      </c>
-      <c r="G6" s="89" t="s">
+    <row r="51" spans="2:8" ht="40" x14ac:dyDescent="0.2">
+      <c r="B51" s="116" t="s">
+        <v>378</v>
+      </c>
+      <c r="C51" s="116" t="s">
         <v>280</v>
       </c>
-      <c r="H6" s="89" t="s">
-        <v>281</v>
-      </c>
-      <c r="I6" s="87" t="s">
-        <v>282</v>
-      </c>
-      <c r="J6" s="89" t="s">
+      <c r="D51" s="116" t="s">
+        <v>354</v>
+      </c>
+      <c r="E51" s="116" t="s">
+        <v>355</v>
+      </c>
+      <c r="F51" s="116" t="s">
+        <v>394</v>
+      </c>
+      <c r="G51" s="117" t="s">
+        <v>402</v>
+      </c>
+      <c r="H51" s="115" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B7" s="88" t="s">
-        <v>284</v>
-      </c>
-      <c r="C7" s="89" t="s">
-        <v>285</v>
-      </c>
-      <c r="D7" s="89" t="s">
-        <v>271</v>
-      </c>
-      <c r="E7" s="89" t="s">
-        <v>279</v>
-      </c>
-      <c r="F7" s="89" t="s">
-        <v>273</v>
-      </c>
-      <c r="G7" s="89" t="s">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B52" s="114" t="s">
+        <v>351</v>
+      </c>
+      <c r="C52" s="114" t="s">
+        <v>269</v>
+      </c>
+      <c r="D52" s="114" t="s">
+        <v>354</v>
+      </c>
+      <c r="E52" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F52" s="114" t="s">
+        <v>395</v>
+      </c>
+      <c r="G52" s="114" t="s">
+        <v>356</v>
+      </c>
+      <c r="H52" s="115" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B53" s="114" t="s">
+        <v>359</v>
+      </c>
+      <c r="C53" s="114" t="s">
+        <v>269</v>
+      </c>
+      <c r="D53" s="114" t="s">
+        <v>354</v>
+      </c>
+      <c r="E53" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F53" s="114" t="s">
+        <v>396</v>
+      </c>
+      <c r="G53" s="114" t="s">
+        <v>360</v>
+      </c>
+      <c r="H53" s="115" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B54" s="114" t="s">
+        <v>376</v>
+      </c>
+      <c r="C54" s="114" t="s">
+        <v>269</v>
+      </c>
+      <c r="D54" s="114" t="s">
+        <v>354</v>
+      </c>
+      <c r="E54" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F54" s="114" t="s">
+        <v>397</v>
+      </c>
+      <c r="G54" s="114" t="s">
+        <v>357</v>
+      </c>
+      <c r="H54" s="115" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B55" s="114" t="s">
+        <v>375</v>
+      </c>
+      <c r="C55" s="114" t="s">
+        <v>269</v>
+      </c>
+      <c r="D55" s="114" t="s">
+        <v>354</v>
+      </c>
+      <c r="E55" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F55" s="114" t="s">
+        <v>395</v>
+      </c>
+      <c r="G55" s="114" t="s">
+        <v>358</v>
+      </c>
+      <c r="H55" s="115" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B56" s="113" t="s">
+        <v>371</v>
+      </c>
+      <c r="C56" s="113"/>
+      <c r="D56" s="113"/>
+      <c r="E56" s="113"/>
+      <c r="F56" s="113"/>
+      <c r="G56" s="113"/>
+      <c r="H56" s="113"/>
+    </row>
+    <row r="57" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B57" s="114" t="s">
+        <v>361</v>
+      </c>
+      <c r="C57" s="114" t="s">
         <v>280</v>
       </c>
-      <c r="H7" s="89" t="s">
-        <v>281</v>
-      </c>
-      <c r="I7" s="87" t="s">
-        <v>282</v>
-      </c>
-      <c r="J7" s="89" t="s">
+      <c r="D57" s="114" t="s">
+        <v>354</v>
+      </c>
+      <c r="E57" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F57" s="114" t="s">
+        <v>393</v>
+      </c>
+      <c r="G57" s="114" t="s">
+        <v>362</v>
+      </c>
+      <c r="H57" s="115" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B8" s="85" t="s">
-        <v>286</v>
-      </c>
-      <c r="C8" s="86" t="s">
-        <v>285</v>
-      </c>
-      <c r="D8" s="86" t="s">
-        <v>271</v>
-      </c>
-      <c r="E8" s="86" t="s">
-        <v>279</v>
-      </c>
-      <c r="F8" s="86" t="s">
-        <v>273</v>
-      </c>
-      <c r="G8" s="86" t="s">
-        <v>287</v>
-      </c>
-      <c r="H8" s="86" t="s">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B58" s="114" t="s">
+        <v>330</v>
+      </c>
+      <c r="C58" s="114" t="s">
+        <v>269</v>
+      </c>
+      <c r="D58" s="114" t="s">
+        <v>354</v>
+      </c>
+      <c r="E58" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F58" s="114" t="s">
+        <v>398</v>
+      </c>
+      <c r="G58" s="114" t="s">
+        <v>363</v>
+      </c>
+      <c r="H58" s="115" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B59" s="113" t="s">
+        <v>364</v>
+      </c>
+      <c r="C59" s="113"/>
+      <c r="D59" s="113"/>
+      <c r="E59" s="113"/>
+      <c r="F59" s="113"/>
+      <c r="G59" s="113"/>
+      <c r="H59" s="113"/>
+    </row>
+    <row r="60" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B60" s="114" t="s">
+        <v>379</v>
+      </c>
+      <c r="C60" s="114" t="s">
+        <v>336</v>
+      </c>
+      <c r="D60" s="114" t="s">
+        <v>365</v>
+      </c>
+      <c r="E60" s="114" t="s">
+        <v>355</v>
+      </c>
+      <c r="F60" s="114" t="s">
+        <v>399</v>
+      </c>
+      <c r="G60" s="114" t="s">
+        <v>366</v>
+      </c>
+      <c r="H60" s="115" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="61" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B61" s="113" t="s">
+        <v>289</v>
+      </c>
+      <c r="C61" s="113"/>
+      <c r="D61" s="113"/>
+      <c r="E61" s="113"/>
+      <c r="F61" s="113"/>
+      <c r="G61" s="113"/>
+      <c r="H61" s="113"/>
+    </row>
+    <row r="62" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B62" s="116" t="s">
+        <v>344</v>
+      </c>
+      <c r="C62" s="116" t="s">
         <v>288</v>
       </c>
-      <c r="I8" s="87" t="s">
-        <v>289</v>
-      </c>
-      <c r="J8" s="89" t="s">
+      <c r="D62" s="116" t="s">
+        <v>365</v>
+      </c>
+      <c r="E62" s="116" t="s">
+        <v>367</v>
+      </c>
+      <c r="F62" s="116" t="s">
+        <v>400</v>
+      </c>
+      <c r="G62" s="116" t="s">
+        <v>382</v>
+      </c>
+      <c r="H62" s="115" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B9" s="85"/>
-      <c r="C9" s="86"/>
-      <c r="D9" s="86"/>
-      <c r="E9" s="86"/>
-      <c r="F9" s="86"/>
-      <c r="G9" s="86"/>
-      <c r="H9" s="86"/>
-      <c r="I9" s="87" t="s">
+    <row r="63" spans="2:8" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H63"/>
+    </row>
+    <row r="64" spans="2:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H64"/>
+    </row>
+    <row r="65" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="H65"/>
+    </row>
+    <row r="66" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B66" s="107"/>
+    </row>
+    <row r="72" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="K72" s="120" t="s">
+        <v>386</v>
+      </c>
+      <c r="L72" s="120"/>
+      <c r="M72" s="120"/>
+      <c r="N72" s="120"/>
+      <c r="O72" s="120"/>
+      <c r="P72" s="120"/>
+    </row>
+    <row r="73" spans="2:16" ht="26" x14ac:dyDescent="0.2">
+      <c r="K73" s="126"/>
+      <c r="L73" s="127"/>
+      <c r="M73" s="128"/>
+      <c r="N73" s="112" t="s">
+        <v>387</v>
+      </c>
+      <c r="O73" s="130" t="s">
+        <v>384</v>
+      </c>
+      <c r="P73" s="112" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="74" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="K74" s="119" t="s">
+        <v>344</v>
+      </c>
+      <c r="L74" s="125" t="s">
+        <v>262</v>
+      </c>
+      <c r="M74" s="118" t="s">
+        <v>288</v>
+      </c>
+      <c r="N74" s="119" t="s">
+        <v>52</v>
+      </c>
+      <c r="O74" s="119" t="s">
+        <v>389</v>
+      </c>
+      <c r="P74" s="121" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="75" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="K75" s="119"/>
+      <c r="L75" s="129" t="s">
+        <v>368</v>
+      </c>
+      <c r="M75" s="117" t="s">
+        <v>365</v>
+      </c>
+      <c r="N75" s="119"/>
+      <c r="O75" s="119"/>
+      <c r="P75" s="121"/>
+    </row>
+    <row r="76" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="K76" s="119"/>
+      <c r="L76" s="129" t="s">
+        <v>265</v>
+      </c>
+      <c r="M76" s="117" t="s">
+        <v>392</v>
+      </c>
+      <c r="N76" s="119"/>
+      <c r="O76" s="119"/>
+      <c r="P76" s="121"/>
+    </row>
+    <row r="77" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="K77" s="119"/>
+      <c r="L77" s="129" t="s">
+        <v>267</v>
+      </c>
+      <c r="M77" s="117" t="s">
         <v>290</v>
       </c>
-      <c r="J9" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B10" s="85"/>
-      <c r="C10" s="86"/>
-      <c r="D10" s="86"/>
-      <c r="E10" s="86"/>
-      <c r="F10" s="86"/>
-      <c r="G10" s="86"/>
-      <c r="H10" s="86"/>
-      <c r="I10" s="87" t="s">
-        <v>291</v>
-      </c>
-      <c r="J10" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B11" s="88" t="s">
-        <v>292</v>
-      </c>
-      <c r="C11" s="89" t="s">
-        <v>270</v>
-      </c>
-      <c r="D11" s="89" t="s">
-        <v>271</v>
-      </c>
-      <c r="E11" s="89" t="s">
-        <v>279</v>
-      </c>
-      <c r="F11" s="89" t="s">
-        <v>273</v>
-      </c>
-      <c r="G11" s="89" t="s">
-        <v>293</v>
-      </c>
-      <c r="H11" s="89" t="s">
-        <v>294</v>
-      </c>
-      <c r="I11" s="87" t="s">
-        <v>295</v>
-      </c>
-      <c r="J11" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B12" s="105" t="s">
-        <v>296</v>
-      </c>
-      <c r="C12" s="89" t="s">
-        <v>297</v>
-      </c>
-      <c r="D12" s="89" t="s">
-        <v>298</v>
-      </c>
-      <c r="E12" s="89" t="s">
-        <v>279</v>
-      </c>
-      <c r="F12" s="89" t="s">
-        <v>273</v>
-      </c>
-      <c r="G12" s="89" t="s">
-        <v>293</v>
-      </c>
-      <c r="H12" s="89" t="s">
-        <v>299</v>
-      </c>
-      <c r="I12" s="87" t="s">
-        <v>300</v>
-      </c>
-      <c r="J12" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B13" s="88" t="s">
-        <v>301</v>
-      </c>
-      <c r="C13" s="89" t="s">
-        <v>270</v>
-      </c>
-      <c r="D13" s="89" t="s">
-        <v>271</v>
-      </c>
-      <c r="E13" s="89" t="s">
-        <v>279</v>
-      </c>
-      <c r="F13" s="89" t="s">
-        <v>273</v>
-      </c>
-      <c r="G13" s="89" t="s">
-        <v>280</v>
-      </c>
-      <c r="H13" s="89" t="s">
-        <v>302</v>
-      </c>
-      <c r="I13" s="87" t="s">
-        <v>303</v>
-      </c>
-      <c r="J13" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B14" s="85" t="s">
-        <v>304</v>
-      </c>
-      <c r="C14" s="86" t="s">
-        <v>285</v>
-      </c>
-      <c r="D14" s="86" t="s">
-        <v>271</v>
-      </c>
-      <c r="E14" s="86" t="s">
-        <v>279</v>
-      </c>
-      <c r="F14" s="86" t="s">
-        <v>273</v>
-      </c>
-      <c r="G14" s="86" t="s">
-        <v>274</v>
-      </c>
-      <c r="H14" s="86" t="s">
-        <v>294</v>
-      </c>
-      <c r="I14" s="87" t="s">
-        <v>305</v>
-      </c>
-      <c r="J14" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B15" s="85"/>
-      <c r="C15" s="86"/>
-      <c r="D15" s="86"/>
-      <c r="E15" s="86"/>
-      <c r="F15" s="86"/>
-      <c r="G15" s="86"/>
-      <c r="H15" s="86"/>
-      <c r="I15" s="87" t="s">
-        <v>306</v>
-      </c>
-      <c r="J15" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B16" s="85" t="s">
-        <v>307</v>
-      </c>
-      <c r="C16" s="86" t="s">
-        <v>285</v>
-      </c>
-      <c r="D16" s="86" t="s">
-        <v>271</v>
-      </c>
-      <c r="E16" s="86" t="s">
-        <v>272</v>
-      </c>
-      <c r="F16" s="86" t="s">
-        <v>273</v>
-      </c>
-      <c r="G16" s="86" t="s">
-        <v>287</v>
-      </c>
-      <c r="H16" s="86" t="s">
-        <v>281</v>
-      </c>
-      <c r="I16" s="87" t="s">
-        <v>308</v>
-      </c>
-      <c r="J16" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B17" s="85"/>
-      <c r="C17" s="86"/>
-      <c r="D17" s="86"/>
-      <c r="E17" s="86"/>
-      <c r="F17" s="86"/>
-      <c r="G17" s="86"/>
-      <c r="H17" s="86"/>
-      <c r="I17" s="87" t="s">
-        <v>309</v>
-      </c>
-      <c r="J17" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B18" s="85"/>
-      <c r="C18" s="86"/>
-      <c r="D18" s="86"/>
-      <c r="E18" s="86"/>
-      <c r="F18" s="86"/>
-      <c r="G18" s="86"/>
-      <c r="H18" s="86"/>
-      <c r="I18" s="87" t="s">
-        <v>310</v>
-      </c>
-      <c r="J18" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B19" s="103" t="s">
-        <v>301</v>
-      </c>
-      <c r="C19" s="90" t="s">
-        <v>270</v>
-      </c>
-      <c r="D19" s="90" t="s">
-        <v>271</v>
-      </c>
-      <c r="E19" s="90" t="s">
-        <v>279</v>
-      </c>
-      <c r="F19" s="90" t="s">
-        <v>273</v>
-      </c>
-      <c r="G19" s="90" t="s">
-        <v>280</v>
-      </c>
-      <c r="H19" s="90" t="s">
-        <v>302</v>
-      </c>
-      <c r="I19" s="91" t="s">
-        <v>311</v>
-      </c>
-      <c r="J19" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B20" s="103"/>
-      <c r="C20" s="90"/>
-      <c r="D20" s="90"/>
-      <c r="E20" s="90"/>
-      <c r="F20" s="90"/>
-      <c r="G20" s="90"/>
-      <c r="H20" s="90"/>
-      <c r="I20" s="91" t="s">
-        <v>312</v>
-      </c>
-      <c r="J20" s="89" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B21" s="104" t="s">
-        <v>292</v>
-      </c>
-      <c r="C21" s="92" t="s">
-        <v>270</v>
-      </c>
-      <c r="D21" s="92" t="s">
-        <v>271</v>
-      </c>
-      <c r="E21" s="92" t="s">
-        <v>279</v>
-      </c>
-      <c r="F21" s="92" t="s">
-        <v>273</v>
-      </c>
-      <c r="G21" s="92" t="s">
-        <v>293</v>
-      </c>
-      <c r="H21" s="92" t="s">
-        <v>294</v>
-      </c>
-      <c r="I21" s="93" t="s">
-        <v>295</v>
-      </c>
-      <c r="J21" s="95" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>314</v>
-      </c>
-      <c r="B25" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B26" s="94" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>315</v>
-      </c>
-      <c r="B27" s="94" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B28" s="94" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B29" s="94" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B35" t="s">
-        <v>339</v>
-      </c>
-      <c r="C35" t="s">
-        <v>340</v>
-      </c>
-      <c r="D35" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="D36" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="C37" t="s">
-        <v>343</v>
-      </c>
-      <c r="D37" t="s">
-        <v>345</v>
-      </c>
-      <c r="E37" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="C38" t="s">
-        <v>252</v>
-      </c>
+      <c r="N77" s="119"/>
+      <c r="O77" s="119"/>
+      <c r="P77" s="121"/>
+    </row>
+    <row r="78" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="K78" s="119"/>
+      <c r="L78" s="129" t="s">
+        <v>353</v>
+      </c>
+      <c r="M78" s="117" t="s">
+        <v>382</v>
+      </c>
+      <c r="N78" s="119"/>
+      <c r="O78" s="119"/>
+      <c r="P78" s="121"/>
+    </row>
+    <row r="79" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="K79" s="122" t="s">
+        <v>373</v>
+      </c>
+      <c r="L79" s="125" t="s">
+        <v>262</v>
+      </c>
+      <c r="M79" s="118" t="s">
+        <v>369</v>
+      </c>
+      <c r="N79" s="119" t="s">
+        <v>383</v>
+      </c>
+      <c r="O79" s="119" t="s">
+        <v>391</v>
+      </c>
+      <c r="P79" s="121" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="80" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="K80" s="123"/>
+      <c r="L80" s="129" t="s">
+        <v>368</v>
+      </c>
+      <c r="M80" s="117" t="s">
+        <v>354</v>
+      </c>
+      <c r="N80" s="119"/>
+      <c r="O80" s="119"/>
+      <c r="P80" s="121"/>
+    </row>
+    <row r="81" spans="11:16" x14ac:dyDescent="0.2">
+      <c r="K81" s="123"/>
+      <c r="L81" s="129" t="s">
+        <v>265</v>
+      </c>
+      <c r="M81" s="117" t="s">
+        <v>390</v>
+      </c>
+      <c r="N81" s="119"/>
+      <c r="O81" s="119"/>
+      <c r="P81" s="121"/>
+    </row>
+    <row r="82" spans="11:16" x14ac:dyDescent="0.2">
+      <c r="K82" s="123"/>
+      <c r="L82" s="129" t="s">
+        <v>267</v>
+      </c>
+      <c r="M82" s="117" t="s">
+        <v>372</v>
+      </c>
+      <c r="N82" s="119"/>
+      <c r="O82" s="119"/>
+      <c r="P82" s="121"/>
+    </row>
+    <row r="83" spans="11:16" x14ac:dyDescent="0.2">
+      <c r="K83" s="124"/>
+      <c r="L83" s="129" t="s">
+        <v>353</v>
+      </c>
+      <c r="M83" s="117" t="s">
+        <v>388</v>
+      </c>
+      <c r="N83" s="119"/>
+      <c r="O83" s="119"/>
+      <c r="P83" s="121"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="G14:G15"/>
+  <mergeCells count="57">
+    <mergeCell ref="K73:M73"/>
+    <mergeCell ref="N79:N83"/>
+    <mergeCell ref="P74:P78"/>
+    <mergeCell ref="P79:P83"/>
+    <mergeCell ref="O74:O78"/>
+    <mergeCell ref="O79:O83"/>
+    <mergeCell ref="K79:K83"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="K72:P72"/>
+    <mergeCell ref="K74:K78"/>
+    <mergeCell ref="N74:N78"/>
+    <mergeCell ref="B47:H47"/>
+    <mergeCell ref="B56:H56"/>
+    <mergeCell ref="B59:H59"/>
+    <mergeCell ref="B61:H61"/>
+    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="F13:F15"/>
+    <mergeCell ref="G13:G15"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="F18:F19"/>
     <mergeCell ref="H3:H4"/>
-    <mergeCell ref="B8:B10"/>
     <mergeCell ref="C8:C10"/>
     <mergeCell ref="D8:D10"/>
     <mergeCell ref="E8:E10"/>
     <mergeCell ref="F8:F10"/>
     <mergeCell ref="G8:G10"/>
     <mergeCell ref="H8:H10"/>
-    <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>

</xml_diff>